<commit_message>
保存: D13 第二步完成, 亮起 12.4 s / 找板 19.8–20.9 s
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/progress/显性目的进度_2026-10-14.xlsx
+++ b/docs/progress/显性目的进度_2026-10-14.xlsx
@@ -15,7 +15,7 @@
     <sheet name="历史记录" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'历史记录'!$A$1:$I$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'历史记录'!$A$1:$I$74</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -231,14 +231,14 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -8335,16 +8335,16 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>0.7567567567567568</v>
+        <v>0.7837837837837838</v>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>28/37</t>
+          <t>29/37</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>KR 18/25 + 交付 10/12 — 统一口径：达成率_P = (P 目标已达标的 KR 数 + P 需要的交付里已完成数) ÷ (有 P 目标的 KR 数 + P 需要的交付总数)，P = V0 / V1 / V2。</t>
+          <t>KR 19/25 + 交付 10/12 — 统一口径：达成率_P = (P 目标已达标的 KR 数 + P 需要的交付里已完成数) ÷ (有 P 目标的 KR 数 + P 需要的交付总数)，P = V0 / V1 / V2。</t>
         </is>
       </c>
       <c r="G4" s="8" t="n">
@@ -8367,16 +8367,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>24/45</t>
+          <t>25/45</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>KR 10/24 + 交付 14/21 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
+          <t>KR 11/24 + 交付 14/21 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
         </is>
       </c>
       <c r="G5" s="8" t="n">
@@ -8399,29 +8399,29 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.4693877551020408</v>
+        <v>0.4897959183673469</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>23/49</t>
+          <t>24/49</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>KR 9/24 + 交付 14/25 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
+          <t>KR 10/24 + 交付 14/25 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
         </is>
       </c>
       <c r="G6" s="8" t="n">
         <v>46309</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>0.7568</v>
+        <v>0.7838000000000001</v>
       </c>
       <c r="I6" s="9" t="n">
-        <v>0.5333</v>
+        <v>0.5556</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>0.4694</v>
+        <v>0.4898</v>
       </c>
     </row>
     <row r="8">
@@ -8540,29 +8540,29 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>KR8.1</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>变差</t>
-        </is>
-      </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>变好</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>上电到 0° 片亮起 (停转) (s, 越小越好)</t>
         </is>
       </c>
-      <c r="D13" s="15" t="inlineStr">
-        <is>
-          <t>15.8 (10-13) → 17.2</t>
-        </is>
-      </c>
-      <c r="E13" s="15" t="inlineStr">
-        <is>
-          <t>12 / 12 / 12；dr1v90 task/d18-pl-default d35c6d4 (上板 3 次重启 17.17–17.30 s)</t>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>15.8 (10-13) → 12.4</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>12 / 12 / 12；dr1v90 d13_boot/runs/20261014_145507 (串口 3 次)</t>
         </is>
       </c>
     </row>
@@ -8584,12 +8584,12 @@
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>25.6 (10-13) → 24.4</t>
+          <t>25.6 (10-13) → 19.8</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>20 / 20 / 20；dr1v90 task/d18-pl-default d35c6d4</t>
+          <t>20 / 20 / 20；dr1v90 d13_boot/runs/20261014_145507</t>
         </is>
       </c>
     </row>
@@ -8714,9 +8714,9 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>🔄</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -8726,7 +8726,7 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>KR8.1;KR8.2;D13 (0/3)</t>
+          <t>KR8.1;KR8.2;D13 (1/3)</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -9219,30 +9219,30 @@
           <t>开</t>
         </is>
       </c>
-      <c r="C43" s="15" t="inlineStr">
+      <c r="C43" s="17" t="inlineStr">
         <is>
           <t>1.2G 可能过不了</t>
         </is>
       </c>
-      <c r="D43" s="15" t="inlineStr">
+      <c r="D43" s="17" t="inlineStr">
         <is>
           <t>影响：DR1 无 SERDES，09-22 DR1↔DR1 1.2G 全死
 应对：退路 1.0G × 16 lane；V1 回板 PRBS 实测定</t>
         </is>
       </c>
-      <c r="E43" s="15" t="inlineStr">
+      <c r="E43" s="17" t="inlineStr">
         <is>
           <t>主会话+硬件 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="17" t="inlineStr">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B44" s="17" t="inlineStr">
+      <c r="B44" s="15" t="inlineStr">
         <is>
           <t>监控</t>
         </is>
@@ -9275,18 +9275,18 @@
           <t>开</t>
         </is>
       </c>
-      <c r="C45" s="15" t="inlineStr">
+      <c r="C45" s="17" t="inlineStr">
         <is>
           <t>灯板 SDO→SDI 0Ω 在 09-18 图上悬空</t>
         </is>
       </c>
-      <c r="D45" s="15" t="inlineStr">
+      <c r="D45" s="17" t="inlineStr">
         <is>
           <t>影响：每块下半屏黑
 应对：硬件确认并补 0Ω</t>
         </is>
       </c>
-      <c r="E45" s="15" t="inlineStr">
+      <c r="E45" s="17" t="inlineStr">
         <is>
           <t>硬件 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
@@ -9303,18 +9303,18 @@
           <t>开</t>
         </is>
       </c>
-      <c r="C46" s="15" t="inlineStr">
+      <c r="C46" s="17" t="inlineStr">
         <is>
           <t>2260 从未收到合法 ACK（疑物理通路）</t>
         </is>
       </c>
-      <c r="D46" s="15" t="inlineStr">
+      <c r="D46" s="17" t="inlineStr">
         <is>
           <t>影响：1 期显示可能起不来
 应对：验证板一颗一组针对此问题，回板验证</t>
         </is>
       </c>
-      <c r="E46" s="15" t="inlineStr">
+      <c r="E46" s="17" t="inlineStr">
         <is>
           <t>硬件+主会话 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
@@ -9331,18 +9331,18 @@
           <t>开</t>
         </is>
       </c>
-      <c r="C47" s="15" t="inlineStr">
+      <c r="C47" s="17" t="inlineStr">
         <is>
           <t>2 期 DDR 带宽：16 bit 余量约 11%，32 bit 像素超限</t>
         </is>
       </c>
-      <c r="D47" s="15" t="inlineStr">
+      <c r="D47" s="17" t="inlineStr">
         <is>
           <t>影响：2 期 32 bit 像素带宽不够
 应对：B 线 T2 板 32 bit DDR + PL 读口 ≥200 MHz/分端口</t>
         </is>
       </c>
-      <c r="E47" s="15" t="inlineStr">
+      <c r="E47" s="17" t="inlineStr">
         <is>
           <t>硬件 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
@@ -9359,30 +9359,30 @@
           <t>开</t>
         </is>
       </c>
-      <c r="C48" s="15" t="inlineStr">
+      <c r="C48" s="17" t="inlineStr">
         <is>
           <t>偶发慢读 133 µs &gt; 30 Hz 片窗 110 µs</t>
         </is>
       </c>
-      <c r="D48" s="15" t="inlineStr">
+      <c r="D48" s="17" t="inlineStr">
         <is>
           <t>影响：偶发迟到掉片
 应对：D16 预取缓冲 + 降争用</t>
         </is>
       </c>
-      <c r="E48" s="15" t="inlineStr">
+      <c r="E48" s="17" t="inlineStr">
         <is>
           <t>主会话 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="17" t="inlineStr">
+      <c r="A49" s="15" t="inlineStr">
         <is>
           <t>R7</t>
         </is>
       </c>
-      <c r="B49" s="17" t="inlineStr">
+      <c r="B49" s="15" t="inlineStr">
         <is>
           <t>监控</t>
         </is>
@@ -9415,30 +9415,30 @@
           <t>开</t>
         </is>
       </c>
-      <c r="C50" s="15" t="inlineStr">
+      <c r="C50" s="17" t="inlineStr">
         <is>
           <t>转子离心 68–136 g：FS03 0.5 mm 板对板、TF 卡</t>
         </is>
       </c>
-      <c r="D50" s="15" t="inlineStr">
+      <c r="D50" s="17" t="inlineStr">
         <is>
           <t>影响：高速下接触不良/脱落
 应对：T2 板留 eMMC、打胶</t>
         </is>
       </c>
-      <c r="E50" s="15" t="inlineStr">
+      <c r="E50" s="17" t="inlineStr">
         <is>
           <t>硬件 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="17" t="inlineStr">
+      <c r="A51" s="15" t="inlineStr">
         <is>
           <t>R9</t>
         </is>
       </c>
-      <c r="B51" s="17" t="inlineStr">
+      <c r="B51" s="15" t="inlineStr">
         <is>
           <t>监控</t>
         </is>
@@ -9471,18 +9471,18 @@
           <t>开</t>
         </is>
       </c>
-      <c r="C52" s="15" t="inlineStr">
+      <c r="C52" s="17" t="inlineStr">
         <is>
           <t>1 期面板映射缺 4 项信息</t>
         </is>
       </c>
-      <c r="D52" s="15" t="inlineStr">
+      <c r="D52" s="17" t="inlineStr">
         <is>
           <t>影响：1 期桥表无法定稿
 应对：问硬件同事</t>
         </is>
       </c>
-      <c r="E52" s="15" t="inlineStr">
+      <c r="E52" s="17" t="inlineStr">
         <is>
           <t>硬件 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
@@ -9576,7 +9576,7 @@
       <c r="A58" s="19" t="n">
         <v>46309</v>
       </c>
-      <c r="B58" s="17" t="inlineStr">
+      <c r="B58" s="15" t="inlineStr">
         <is>
           <t>问题</t>
         </is>
@@ -9601,7 +9601,7 @@
       <c r="A59" s="19" t="n">
         <v>46309</v>
       </c>
-      <c r="B59" s="17" t="inlineStr">
+      <c r="B59" s="15" t="inlineStr">
         <is>
           <t>问题</t>
         </is>
@@ -9651,7 +9651,7 @@
       <c r="A61" s="19" t="n">
         <v>46309</v>
       </c>
-      <c r="B61" s="17" t="inlineStr">
+      <c r="B61" s="15" t="inlineStr">
         <is>
           <t>问题</t>
         </is>
@@ -9726,7 +9726,7 @@
       <c r="A64" s="19" t="n">
         <v>46309</v>
       </c>
-      <c r="B64" s="17" t="inlineStr">
+      <c r="B64" s="15" t="inlineStr">
         <is>
           <t>问题</t>
         </is>
@@ -9976,7 +9976,7 @@
       <c r="A74" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B74" s="17" t="inlineStr">
+      <c r="B74" s="15" t="inlineStr">
         <is>
           <t>问题</t>
         </is>
@@ -10101,7 +10101,7 @@
       <c r="A79" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B79" s="17" t="inlineStr">
+      <c r="B79" s="15" t="inlineStr">
         <is>
           <t>问题</t>
         </is>
@@ -10126,7 +10126,7 @@
       <c r="A80" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B80" s="17" t="inlineStr">
+      <c r="B80" s="15" t="inlineStr">
         <is>
           <t>问题</t>
         </is>
@@ -10276,7 +10276,7 @@
       <c r="A86" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B86" s="17" t="inlineStr">
+      <c r="B86" s="15" t="inlineStr">
         <is>
           <t>问题</t>
         </is>
@@ -10351,7 +10351,7 @@
       <c r="A89" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B89" s="17" t="inlineStr">
+      <c r="B89" s="15" t="inlineStr">
         <is>
           <t>问题</t>
         </is>
@@ -10639,7 +10639,7 @@
       <c r="A101" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B101" s="17" t="inlineStr">
+      <c r="B101" s="15" t="inlineStr">
         <is>
           <t>问题</t>
         </is>
@@ -11786,7 +11786,7 @@
           <t>稳定</t>
         </is>
       </c>
-      <c r="D19" s="17" t="inlineStr">
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t>🔄 进行中 / 未达标</t>
         </is>
@@ -11890,7 +11890,7 @@
       <c r="N20" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="O20" s="17" t="inlineStr">
+      <c r="O20" s="15" t="inlineStr">
         <is>
           <t>🔄</t>
         </is>
@@ -11963,7 +11963,7 @@
           <t>运维</t>
         </is>
       </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="D22" s="15" t="inlineStr">
         <is>
           <t>🔄 进行中 / 未达标</t>
         </is>
@@ -11989,7 +11989,7 @@
         </is>
       </c>
       <c r="I22" s="6" t="n">
-        <v>17.2</v>
+        <v>12.4</v>
       </c>
       <c r="J22" s="19" t="n">
         <v>46309</v>
@@ -12008,18 +12008,18 @@
       <c r="N22" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="O22" s="17" t="inlineStr">
+      <c r="O22" s="15" t="inlineStr">
         <is>
           <t>🔄</t>
         </is>
       </c>
       <c r="P22" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d18-pl-default d35c6d4 (上板 3 次重启 17.17–17.30 s)</t>
+          <t>dr1v90 d13_boot/runs/20261014_145507 (串口 3 次)</t>
         </is>
       </c>
       <c r="Q22" s="23" t="n">
-        <v>0.6976744186046512</v>
+        <v>0.9677419354838709</v>
       </c>
     </row>
     <row r="23">
@@ -12061,7 +12061,7 @@
       <c r="L23" s="6" t="n"/>
       <c r="M23" s="6" t="n"/>
       <c r="N23" s="6" t="n"/>
-      <c r="O23" s="17" t="inlineStr">
+      <c r="O23" s="15" t="inlineStr">
         <is>
           <t>🔄</t>
         </is>
@@ -12099,7 +12099,7 @@
         </is>
       </c>
       <c r="I24" s="6" t="n">
-        <v>24.4</v>
+        <v>19.8</v>
       </c>
       <c r="J24" s="19" t="n">
         <v>46309</v>
@@ -12118,18 +12118,18 @@
       <c r="N24" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="O24" s="17" t="inlineStr">
-        <is>
-          <t>🔄</t>
+      <c r="O24" s="14" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="P24" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d18-pl-default d35c6d4</t>
+          <t>dr1v90 d13_boot/runs/20261014_145507</t>
         </is>
       </c>
       <c r="Q24" s="23" t="n">
-        <v>0.819672131147541</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -12205,7 +12205,7 @@
           <t>运维</t>
         </is>
       </c>
-      <c r="D26" s="17" t="inlineStr">
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>🔄 进行中 / 未达标</t>
         </is>
@@ -12250,7 +12250,7 @@
       <c r="N26" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O26" s="17" t="inlineStr">
+      <c r="O26" s="15" t="inlineStr">
         <is>
           <t>🔄</t>
         </is>
@@ -12309,7 +12309,7 @@
       <c r="N27" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O27" s="17" t="inlineStr">
+      <c r="O27" s="15" t="inlineStr">
         <is>
           <t>🔄</t>
         </is>
@@ -12475,7 +12475,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="17" t="inlineStr">
+      <c r="A33" s="15" t="inlineStr">
         <is>
           <t>🔄</t>
         </is>
@@ -14557,7 +14557,7 @@
         <v>46309</v>
       </c>
       <c r="B295" s="6" t="n">
-        <v>17.2</v>
+        <v>12.4</v>
       </c>
       <c r="C295" s="6" t="n"/>
       <c r="D295" s="8" t="n">
@@ -14698,7 +14698,7 @@
         <v>46309</v>
       </c>
       <c r="B329" s="6" t="n">
-        <v>24.4</v>
+        <v>19.8</v>
       </c>
       <c r="C329" s="6" t="n"/>
       <c r="D329" s="8" t="n">
@@ -16010,7 +16010,7 @@
         <v>46312</v>
       </c>
       <c r="F38" s="19" t="n"/>
-      <c r="G38" s="17" t="inlineStr">
+      <c r="G38" s="15" t="inlineStr">
         <is>
           <t>🔄</t>
         </is>
@@ -16190,7 +16190,7 @@
         <v>46310</v>
       </c>
       <c r="F43" s="19" t="n"/>
-      <c r="G43" s="17" t="inlineStr">
+      <c r="G43" s="15" t="inlineStr">
         <is>
           <t>🔄</t>
         </is>
@@ -16226,7 +16226,7 @@
         <v>46311</v>
       </c>
       <c r="F44" s="19" t="n"/>
-      <c r="G44" s="17" t="inlineStr">
+      <c r="G44" s="15" t="inlineStr">
         <is>
           <t>🔄</t>
         </is>
@@ -16262,7 +16262,7 @@
         <v>46311</v>
       </c>
       <c r="F45" s="19" t="n"/>
-      <c r="G45" s="17" t="inlineStr">
+      <c r="G45" s="15" t="inlineStr">
         <is>
           <t>🔄</t>
         </is>
@@ -16298,7 +16298,7 @@
         <v>46312</v>
       </c>
       <c r="F46" s="19" t="n"/>
-      <c r="G46" s="17" t="inlineStr">
+      <c r="G46" s="15" t="inlineStr">
         <is>
           <t>🔄</t>
         </is>
@@ -16334,7 +16334,7 @@
         <v>46312</v>
       </c>
       <c r="F47" s="19" t="n"/>
-      <c r="G47" s="17" t="inlineStr">
+      <c r="G47" s="15" t="inlineStr">
         <is>
           <t>🔄</t>
         </is>
@@ -16651,7 +16651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -19591,40 +19591,122 @@
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
+          <t>KR8.1</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>上电到 0° 片亮起 (停转)</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>V0 2047</t>
+        </is>
+      </c>
+      <c r="H72" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 d13_boot/runs/20261014_145507 (串口 3 次)</t>
+        </is>
+      </c>
+      <c r="I72" s="7" t="inlineStr">
+        <is>
+          <t>D13 第二步后 (bootdelay 0 + 精简 uInitrd) + PL 默认开机</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="31" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B73" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
           <t>KR8.2</t>
         </is>
       </c>
-      <c r="D72" s="7" t="inlineStr">
+      <c r="D73" s="7" t="inlineStr">
         <is>
           <t>按名字找到板子</t>
         </is>
       </c>
-      <c r="E72" s="7" t="inlineStr">
+      <c r="E73" s="7" t="inlineStr">
         <is>
           <t>s</t>
         </is>
       </c>
-      <c r="F72" s="7" t="n">
+      <c r="F73" s="7" t="n">
         <v>24.4</v>
       </c>
-      <c r="G72" s="7" t="inlineStr">
+      <c r="G73" s="7" t="inlineStr">
         <is>
           <t>V0 2047</t>
         </is>
       </c>
-      <c r="H72" s="7" t="inlineStr">
+      <c r="H73" s="7" t="inlineStr">
         <is>
           <t>dr1v90 task/d18-pl-default d35c6d4</t>
         </is>
       </c>
-      <c r="I72" s="7" t="inlineStr">
+      <c r="I73" s="7" t="inlineStr">
         <is>
           <t>PL 默认开机找板 24.4–28.3 s</t>
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" s="31" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B74" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>KR8.2</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>按名字找到板子</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>V0 2047</t>
+        </is>
+      </c>
+      <c r="H74" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 d13_boot/runs/20261014_145507</t>
+        </is>
+      </c>
+      <c r="I74" s="7" t="inlineStr">
+        <is>
+          <t>3 次 19.8/20.3/20.9 s</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I72"/>
+  <autoFilter ref="A1:I74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[进度] D7 合主线 dee9be6, V0 出口 ⑤ 达成 (6/8); D15b 根因记录
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/progress/显性目的进度_2026-10-14.xlsx
+++ b/docs/progress/显性目的进度_2026-10-14.xlsx
@@ -15,7 +15,7 @@
     <sheet name="历史记录" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'历史记录'!$A$1:$I$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'历史记录'!$A$1:$I$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -4099,12 +4099,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'指标趋势'!$A$362</f>
+              <f>'指标趋势'!$A$362:$A$363</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'指标趋势'!$B$362</f>
+              <f>'指标趋势'!$B$362:$B$363</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -4225,7 +4225,7 @@
         <scaling>
           <orientation val="minMax"/>
           <max val="46309"/>
-          <min val="46307"/>
+          <min val="46308"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -4341,12 +4341,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'指标趋势'!$A$379</f>
+              <f>'指标趋势'!$A$379:$A$380</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'指标趋势'!$B$379</f>
+              <f>'指标趋势'!$B$379:$B$380</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -4467,7 +4467,7 @@
         <scaling>
           <orientation val="minMax"/>
           <max val="46309"/>
-          <min val="46307"/>
+          <min val="46308"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -8264,7 +8264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J103"/>
+  <dimension ref="A1:J107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8335,16 +8335,16 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>0.8378378378378378</v>
+        <v>0.918918918918919</v>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>31/37</t>
+          <t>34/37</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>KR 20/25 + 交付 11/12 — 统一口径：达成率_P = (P 目标已达标的 KR 数 + P 需要的交付里已完成数) ÷ (有 P 目标的 KR 数 + P 需要的交付总数)，P = V0 / V1 / V2。</t>
+          <t>KR 22/25 + 交付 12/12 — 统一口径：达成率_P = (P 目标已达标的 KR 数 + P 需要的交付里已完成数) ÷ (有 P 目标的 KR 数 + P 需要的交付总数)，P = V0 / V1 / V2。</t>
         </is>
       </c>
       <c r="G4" s="8" t="n">
@@ -8367,16 +8367,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0.6</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>27/45</t>
+          <t>30/45</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>KR 12/24 + 交付 15/21 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
+          <t>KR 14/24 + 交付 16/21 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
         </is>
       </c>
       <c r="G5" s="8" t="n">
@@ -8399,29 +8399,29 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.5306122448979592</v>
+        <v>0.5918367346938775</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>26/49</t>
+          <t>29/49</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>KR 11/24 + 交付 15/25 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
+          <t>KR 13/24 + 交付 16/25 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
         </is>
       </c>
       <c r="G6" s="8" t="n">
         <v>46309</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>0.8378</v>
+        <v>0.9189000000000001</v>
       </c>
       <c r="I6" s="9" t="n">
-        <v>0.6</v>
+        <v>0.6667</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>0.5306</v>
+        <v>0.5918</v>
       </c>
     </row>
     <row r="8">
@@ -8593,98 +8593,98 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>KR9.1</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>变好</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>转子遥测可用 (1=可用) (是/否, 越大越好)</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>0 (10-13) → 1</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>1 / 1 / 1；dr1v90 dee9be6</t>
+        </is>
+      </c>
+    </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>阶段出口清单 — V0 出口  (已打勾 5/8；状态由关联项在当日是否完成/达标推出)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>KR9.2</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>变好</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>远程升级失败自动回滚 (1=有) (是/否, 越大越好)</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>0 (10-13) → 1</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>1 / 1 / 1；dr1v90 dee9be6</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>阶段出口清单 — V0 出口  (已打勾 6/8；状态由关联项在当日是否完成/达标推出)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>条目</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>关联项进度</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>来源</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>①2047 PL 切片上板通过</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>D2 (1/1)</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>10-13 主会话规划</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>②主机实时推流 15 fps</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>D1 (1/1)</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>10-13 主会话规划</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -8694,12 +8694,12 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>③几何更正 + 镜像已核实</t>
+          <t>①2047 PL 切片上板通过</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>KR5.2 (1/1)</t>
+          <t>D2 (1/1)</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
@@ -8711,7 +8711,7 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
@@ -8721,12 +8721,12 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>④复位到亮起 ≤12 s、找板 ≤20 s</t>
+          <t>②主机实时推流 15 fps</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>KR8.1;KR8.2;D13 (3/3)</t>
+          <t>D1 (1/1)</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -8738,22 +8738,22 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>⬜</t>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>⑤无串口远程运维：遥测 + 升级失败自动回滚</t>
+          <t>③几何更正 + 镜像已核实</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>D7;KR9.1;KR9.2 (0/3)</t>
+          <t>KR5.2 (1/1)</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
@@ -8765,22 +8765,22 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>⬜</t>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>⑥软件链路无人值守 ≥8 h</t>
+          <t>④复位到亮起 ≤12 s、找板 ≤20 s</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>KR7.2 (0/1)</t>
+          <t>KR8.1;KR8.2;D13 (3/3)</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
@@ -8792,22 +8792,22 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B24" s="12" t="inlineStr">
-        <is>
-          <t>⬜</t>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>⑦WiFi 端 12-bit 通路在 2047 上跑通</t>
+          <t>⑤无串口远程运维：遥测 + 升级失败自动回滚</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>D15 (0/1)</t>
+          <t>D7;KR9.1;KR9.2 (3/3)</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
@@ -8819,137 +8819,137 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>⑥软件链路无人值守 ≥8 h</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>KR7.2 (0/1)</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>10-13 主会话规划</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>⑦WiFi 端 12-bit 通路在 2047 上跑通</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>D15 (0/1)</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>10-13 主会话规划</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>⑧内容 ≥2 + 一种交互</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>KR10.1;KR10.2 (2/2)</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>10-13 主会话规划</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t>阶段出口清单 — V1 回板当天就绪  (已打勾 3/11；状态由关联项在当日是否完成/达标推出)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>阶段出口清单 — V1 回板当天就绪  (已打勾 4/11；状态由关联项在当日是否完成/达标推出)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>条目</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>关联项进度</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>来源</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B29" s="12" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>①主控 1 期整合位流 (PL 切片 + 12-bit 上行，V3 引脚)</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>D10 (0/1)</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>10-13 主会话规划</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B30" s="14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>②桥 1 期 6 链 24 Hz 位流</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>D5 (1/1)</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>10-13 主会话规划</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B31" s="14" t="inlineStr">
-        <is>
-          <t>✅</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>③桥接收 + 1.2G PRBS 测试件</t>
+          <t>①主控 1 期整合位流 (PL 切片 + 12-bit 上行，V3 引脚)</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>D4 (1/1)</t>
+          <t>D10 (0/1)</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -8961,7 +8961,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
@@ -8971,12 +8971,12 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>④1 期几何 LUT + 校准工具</t>
+          <t>②桥 1 期 6 链 24 Hz 位流</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>D6 (1/1)</t>
+          <t>D5 (1/1)</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
@@ -8988,22 +8988,22 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>⬜</t>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>⑤主控↔桥↔2260 联合仿真 0 错</t>
+          <t>③桥接收 + 1.2G PRBS 测试件</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>D8 (0/1)</t>
+          <t>D4 (1/1)</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -9015,22 +9015,22 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>⬜</t>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>⑥全链路系统仿真</t>
+          <t>④1 期几何 LUT + 校准工具</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>D9 (0/1)</t>
+          <t>D6 (1/1)</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
@@ -9042,7 +9042,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B35" s="12" t="inlineStr">
@@ -9052,12 +9052,12 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>⑦C1 台架逐像素 0 错</t>
+          <t>⑤主控↔桥↔2260 联合仿真 0 错</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>D11 (0/1)</t>
+          <t>D8 (0/1)</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
@@ -9069,7 +9069,7 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B36" s="12" t="inlineStr">
@@ -9079,12 +9079,12 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>⑧整机回板点亮步骤 + 一键脚本</t>
+          <t>⑥全链路系统仿真</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>人工状态</t>
+          <t>D9 (0/1)</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
@@ -9096,7 +9096,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B37" s="12" t="inlineStr">
@@ -9106,12 +9106,12 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>⑨硬件确认清单闭环：灯板 SDO→SDI 0Ω、CN3/CN6 n→n、R176–R181 等</t>
+          <t>⑦C1 台架逐像素 0 错</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>人工状态</t>
+          <t>D11 (0/1)</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
@@ -9123,7 +9123,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B38" s="12" t="inlineStr">
@@ -9133,7 +9133,7 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>⑩面板映射 4 项信息到位</t>
+          <t>⑧整机回板点亮步骤 + 一键脚本</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
@@ -9150,425 +9150,429 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>⑨硬件确认清单闭环：灯板 SDO→SDI 0Ω、CN3/CN6 n→n、R176–R181 等</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>人工状态</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>10-13 主会话规划</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>⑩面板映射 4 项信息到位</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>人工状态</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>10-13 主会话规划</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>⑪无串口运维可用</t>
         </is>
       </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>D7 (0/1)</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr">
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>D7 (1/1)</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
         <is>
           <t>10-13 主会话规划</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="10" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>风险表 (risks.csv；红 = 开，黄 = 监控，绿 = 关)</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>编号</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>风险</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>影响 / 应对</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>负责 · 登记日期 · 来源</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="15" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="15" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="B43" s="15" t="inlineStr">
+      <c r="B45" s="15" t="inlineStr">
         <is>
           <t>开</t>
         </is>
       </c>
-      <c r="C43" s="16" t="inlineStr">
+      <c r="C45" s="16" t="inlineStr">
         <is>
           <t>1.2G 可能过不了</t>
         </is>
       </c>
-      <c r="D43" s="16" t="inlineStr">
+      <c r="D45" s="16" t="inlineStr">
         <is>
           <t>影响：DR1 无 SERDES，09-22 DR1↔DR1 1.2G 全死
 应对：退路 1.0G × 16 lane；V1 回板 PRBS 实测定</t>
         </is>
       </c>
-      <c r="E43" s="16" t="inlineStr">
+      <c r="E45" s="16" t="inlineStr">
         <is>
           <t>主会话+硬件 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="17" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="17" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B44" s="17" t="inlineStr">
+      <c r="B46" s="17" t="inlineStr">
         <is>
           <t>监控</t>
         </is>
       </c>
-      <c r="C44" s="18" t="inlineStr">
+      <c r="C46" s="18" t="inlineStr">
         <is>
           <t>1 期 4,296 片/s 桥链路余量仅 0.40%</t>
         </is>
       </c>
-      <c r="D44" s="18" t="inlineStr">
+      <c r="D46" s="18" t="inlineStr">
         <is>
           <t>影响：时钟偏差会丢帧
 应对：退路降到 22 Hz（用户定保持 24 Hz）</t>
         </is>
       </c>
-      <c r="E44" s="18" t="inlineStr">
+      <c r="E46" s="18" t="inlineStr">
         <is>
           <t>主会话 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="15" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="15" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="B45" s="15" t="inlineStr">
+      <c r="B47" s="15" t="inlineStr">
         <is>
           <t>开</t>
         </is>
       </c>
-      <c r="C45" s="16" t="inlineStr">
+      <c r="C47" s="16" t="inlineStr">
         <is>
           <t>灯板 SDO→SDI 0Ω 在 09-18 图上悬空</t>
         </is>
       </c>
-      <c r="D45" s="16" t="inlineStr">
+      <c r="D47" s="16" t="inlineStr">
         <is>
           <t>影响：每块下半屏黑
 应对：硬件确认并补 0Ω</t>
         </is>
       </c>
-      <c r="E45" s="16" t="inlineStr">
+      <c r="E47" s="16" t="inlineStr">
         <is>
           <t>硬件 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="15" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
         <is>
           <t>R4</t>
         </is>
       </c>
-      <c r="B46" s="15" t="inlineStr">
+      <c r="B48" s="15" t="inlineStr">
         <is>
           <t>开</t>
         </is>
       </c>
-      <c r="C46" s="16" t="inlineStr">
+      <c r="C48" s="16" t="inlineStr">
         <is>
           <t>2260 从未收到合法 ACK（疑物理通路）</t>
         </is>
       </c>
-      <c r="D46" s="16" t="inlineStr">
+      <c r="D48" s="16" t="inlineStr">
         <is>
           <t>影响：1 期显示可能起不来
 应对：验证板一颗一组针对此问题，回板验证</t>
         </is>
       </c>
-      <c r="E46" s="16" t="inlineStr">
+      <c r="E48" s="16" t="inlineStr">
         <is>
           <t>硬件+主会话 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="15" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="15" t="inlineStr">
         <is>
           <t>R5</t>
         </is>
       </c>
-      <c r="B47" s="15" t="inlineStr">
+      <c r="B49" s="15" t="inlineStr">
         <is>
           <t>开</t>
         </is>
       </c>
-      <c r="C47" s="16" t="inlineStr">
+      <c r="C49" s="16" t="inlineStr">
         <is>
           <t>2 期 DDR 带宽：16 bit 余量约 11%，32 bit 像素超限</t>
         </is>
       </c>
-      <c r="D47" s="16" t="inlineStr">
+      <c r="D49" s="16" t="inlineStr">
         <is>
           <t>影响：2 期 32 bit 像素带宽不够
 应对：B 线 T2 板 32 bit DDR + PL 读口 ≥200 MHz/分端口</t>
         </is>
       </c>
-      <c r="E47" s="16" t="inlineStr">
+      <c r="E49" s="16" t="inlineStr">
         <is>
           <t>硬件 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="15" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="15" t="inlineStr">
         <is>
           <t>R6</t>
         </is>
       </c>
-      <c r="B48" s="15" t="inlineStr">
+      <c r="B50" s="15" t="inlineStr">
         <is>
           <t>开</t>
         </is>
       </c>
-      <c r="C48" s="16" t="inlineStr">
+      <c r="C50" s="16" t="inlineStr">
         <is>
           <t>偶发慢读 133 µs &gt; 30 Hz 片窗 110 µs</t>
         </is>
       </c>
-      <c r="D48" s="16" t="inlineStr">
+      <c r="D50" s="16" t="inlineStr">
         <is>
           <t>影响：偶发迟到掉片
 应对：D16 预取缓冲 + 降争用</t>
         </is>
       </c>
-      <c r="E48" s="16" t="inlineStr">
+      <c r="E50" s="16" t="inlineStr">
         <is>
           <t>主会话 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="17" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
         <is>
           <t>R7</t>
         </is>
       </c>
-      <c r="B49" s="17" t="inlineStr">
+      <c r="B51" s="17" t="inlineStr">
         <is>
           <t>监控</t>
         </is>
       </c>
-      <c r="C49" s="18" t="inlineStr">
+      <c r="C51" s="18" t="inlineStr">
         <is>
           <t>WiFi/主机负载造成延迟尾巴（10-13 晚 p99 334 ms）</t>
         </is>
       </c>
-      <c r="D49" s="18" t="inlineStr">
+      <c r="D51" s="18" t="inlineStr">
         <is>
           <t>影响：延迟抖动超标
 应对：演示时停重任务；后续增量帧</t>
         </is>
       </c>
-      <c r="E49" s="18" t="inlineStr">
+      <c r="E51" s="18" t="inlineStr">
         <is>
           <t>主会话 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="15" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="15" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
-      <c r="B50" s="15" t="inlineStr">
+      <c r="B52" s="15" t="inlineStr">
         <is>
           <t>开</t>
         </is>
       </c>
-      <c r="C50" s="16" t="inlineStr">
+      <c r="C52" s="16" t="inlineStr">
         <is>
           <t>转子离心 68–136 g：FS03 0.5 mm 板对板、TF 卡</t>
         </is>
       </c>
-      <c r="D50" s="16" t="inlineStr">
+      <c r="D52" s="16" t="inlineStr">
         <is>
           <t>影响：高速下接触不良/脱落
 应对：T2 板留 eMMC、打胶</t>
         </is>
       </c>
-      <c r="E50" s="16" t="inlineStr">
+      <c r="E52" s="16" t="inlineStr">
         <is>
           <t>硬件 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="17" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
         <is>
           <t>R9</t>
         </is>
       </c>
-      <c r="B51" s="17" t="inlineStr">
+      <c r="B53" s="17" t="inlineStr">
         <is>
           <t>监控</t>
         </is>
       </c>
-      <c r="C51" s="18" t="inlineStr">
+      <c r="C53" s="18" t="inlineStr">
         <is>
           <t>D 盘 EIO（IP-guard 驱动）</t>
         </is>
       </c>
-      <c r="D51" s="18" t="inlineStr">
+      <c r="D53" s="18" t="inlineStr">
         <is>
           <t>影响：构建/提交偶发失败
 应对：看门狗自动重挂 + 构建放 WSL 本地盘</t>
         </is>
       </c>
-      <c r="E51" s="18" t="inlineStr">
+      <c r="E53" s="18" t="inlineStr">
         <is>
           <t>主会话 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="15" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="15" t="inlineStr">
         <is>
           <t>R10</t>
         </is>
       </c>
-      <c r="B52" s="15" t="inlineStr">
+      <c r="B54" s="15" t="inlineStr">
         <is>
           <t>开</t>
         </is>
       </c>
-      <c r="C52" s="16" t="inlineStr">
+      <c r="C54" s="16" t="inlineStr">
         <is>
           <t>1 期面板映射缺 4 项信息</t>
         </is>
       </c>
-      <c r="D52" s="16" t="inlineStr">
+      <c r="D54" s="16" t="inlineStr">
         <is>
           <t>影响：1 期桥表无法定稿
 应对：问硬件同事</t>
         </is>
       </c>
-      <c r="E52" s="16" t="inlineStr">
+      <c r="E54" s="16" t="inlineStr">
         <is>
           <t>硬件 · 2026-10-13 · 10-13 主会话规划</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="10" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
         <is>
           <t>每日流水 (daily_log.csv，按天倒序)</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>类型</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>编号</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>来源</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="19" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B56" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
-        </is>
-      </c>
-      <c r="C56" s="7" t="inlineStr">
-        <is>
-          <t>D3</t>
-        </is>
-      </c>
-      <c r="D56" s="7" t="inlineStr">
-        <is>
-          <t>上行出口全量复验 45/0, 合主线</t>
-        </is>
-      </c>
-      <c r="E56" s="7" t="inlineStr">
-        <is>
-          <t>dr1v90 fdb4de6</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="19" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B57" s="15" t="inlineStr">
-        <is>
-          <t>复验退回</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="inlineStr">
-        <is>
-          <t>D2</t>
-        </is>
-      </c>
-      <c r="D57" s="7" t="inlineStr">
-        <is>
-          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
-        </is>
-      </c>
-      <c r="E57" s="7" t="inlineStr">
-        <is>
-          <t>scratchpad/v_pls4_board.log</t>
         </is>
       </c>
     </row>
@@ -9576,24 +9580,24 @@
       <c r="A58" s="19" t="n">
         <v>46309</v>
       </c>
-      <c r="B58" s="17" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B58" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
+          <t>上行出口全量复验 45/0, 合主线</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>dr1v90 fdb4de6</t>
         </is>
       </c>
     </row>
@@ -9601,24 +9605,24 @@
       <c r="A59" s="19" t="n">
         <v>46309</v>
       </c>
-      <c r="B59" s="17" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B59" s="15" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
+          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>scratchpad/v_pls4_board.log</t>
         </is>
       </c>
     </row>
@@ -9626,24 +9630,24 @@
       <c r="A60" s="19" t="n">
         <v>46309</v>
       </c>
-      <c r="B60" s="20" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B60" s="17" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
+          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>project_short_term_delivery_1013</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -9658,17 +9662,17 @@
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
+          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 debd3cd</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -9676,24 +9680,24 @@
       <c r="A62" s="19" t="n">
         <v>46309</v>
       </c>
-      <c r="B62" s="15" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B62" s="20" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
+          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>scratchpad v_pls6_board.log</t>
+          <t>project_short_term_delivery_1013</t>
         </is>
       </c>
     </row>
@@ -9701,9 +9705,9 @@
       <c r="A63" s="19" t="n">
         <v>46309</v>
       </c>
-      <c r="B63" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B63" s="17" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
@@ -9713,12 +9717,12 @@
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
+          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>dr1v90 task/pls-2047 debd3cd</t>
         </is>
       </c>
     </row>
@@ -9726,24 +9730,24 @@
       <c r="A64" s="19" t="n">
         <v>46309</v>
       </c>
-      <c r="B64" s="17" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B64" s="15" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
+          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16-ddr 539d303</t>
+          <t>scratchpad v_pls6_board.log</t>
         </is>
       </c>
     </row>
@@ -9751,24 +9755,24 @@
       <c r="A65" s="19" t="n">
         <v>46309</v>
       </c>
-      <c r="B65" s="20" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B65" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
+          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>feedback_save_weekly_quota</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -9776,24 +9780,24 @@
       <c r="A66" s="19" t="n">
         <v>46309</v>
       </c>
-      <c r="B66" s="21" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B66" s="17" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
+          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>dr1v90 task/d16-ddr 539d303</t>
         </is>
       </c>
     </row>
@@ -9801,24 +9805,24 @@
       <c r="A67" s="19" t="n">
         <v>46309</v>
       </c>
-      <c r="B67" s="14" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B67" s="20" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
+          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 2364e5c</t>
+          <t>feedback_save_weekly_quota</t>
         </is>
       </c>
     </row>
@@ -9833,17 +9837,17 @@
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
+          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>用户在场实转</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -9851,24 +9855,24 @@
       <c r="A69" s="19" t="n">
         <v>46309</v>
       </c>
-      <c r="B69" s="20" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B69" s="14" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
+          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 2364e5c</t>
         </is>
       </c>
     </row>
@@ -9876,24 +9880,24 @@
       <c r="A70" s="19" t="n">
         <v>46309</v>
       </c>
-      <c r="B70" s="14" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B70" s="21" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
+          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d18-pl-default d35c6d4</t>
+          <t>用户在场实转</t>
         </is>
       </c>
     </row>
@@ -9908,12 +9912,12 @@
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
+          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
@@ -9924,7 +9928,7 @@
     </row>
     <row r="72">
       <c r="A72" s="19" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B72" s="14" t="inlineStr">
         <is>
@@ -9933,48 +9937,48 @@
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
+          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 b0f6b5d</t>
+          <t>dr1v90 task/d18-pl-default d35c6d4</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="19" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B73" s="14" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B73" s="20" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
+          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 71d006f / 473abcf</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="19" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B74" s="14" t="inlineStr">
         <is>
@@ -9983,42 +9987,42 @@
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
+          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 596b191</t>
+          <t>dr1v90 dee9be6</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="19" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B75" s="17" t="inlineStr">
-        <is>
-          <t>问题</t>
+        <v>46309</v>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D15b</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
+          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 60c619a / 596b191</t>
+          <t>dr1v90 task/d15b-color-p2</t>
         </is>
       </c>
     </row>
@@ -10028,22 +10032,22 @@
       </c>
       <c r="B76" s="14" t="inlineStr">
         <is>
-          <t>复验通过</t>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
+          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 9bf16ad</t>
+          <t>dr1v90 b0f6b5d</t>
         </is>
       </c>
     </row>
@@ -10051,24 +10055,24 @@
       <c r="A77" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B77" s="15" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B77" s="14" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
+          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 71d006f / 473abcf</t>
         </is>
       </c>
     </row>
@@ -10078,22 +10082,22 @@
       </c>
       <c r="B78" s="14" t="inlineStr">
         <is>
-          <t>复验通过</t>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
+          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 6a373d3</t>
+          <t>dr1v90 596b191</t>
         </is>
       </c>
     </row>
@@ -10101,24 +10105,24 @@
       <c r="A79" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B79" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B79" s="17" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
+          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 cdf49c6</t>
+          <t>dr1v90 60c619a / 596b191</t>
         </is>
       </c>
     </row>
@@ -10126,24 +10130,24 @@
       <c r="A80" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B80" s="17" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B80" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
+          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 9bf16ad</t>
         </is>
       </c>
     </row>
@@ -10151,19 +10155,19 @@
       <c r="A81" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B81" s="17" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B81" s="15" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
+          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
@@ -10183,17 +10187,17 @@
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
+          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 44ed2cd</t>
+          <t>dr1v90 6a373d3</t>
         </is>
       </c>
     </row>
@@ -10201,24 +10205,24 @@
       <c r="A83" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B83" s="15" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B83" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
+          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 cdf49c6</t>
         </is>
       </c>
     </row>
@@ -10226,24 +10230,24 @@
       <c r="A84" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B84" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B84" s="17" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
+          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ffbfeeb</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -10251,19 +10255,19 @@
       <c r="A85" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B85" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B85" s="17" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
+          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
@@ -10276,24 +10280,24 @@
       <c r="A86" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B86" s="15" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B86" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
+          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 44ed2cd</t>
         </is>
       </c>
     </row>
@@ -10301,24 +10305,24 @@
       <c r="A87" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B87" s="17" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B87" s="15" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
+          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 764f81d</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -10326,24 +10330,24 @@
       <c r="A88" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B88" s="15" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B88" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
+          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 ffbfeeb</t>
         </is>
       </c>
     </row>
@@ -10351,24 +10355,24 @@
       <c r="A89" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B89" s="21" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B89" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
+          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d13-boot fdbb217</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -10376,19 +10380,19 @@
       <c r="A90" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B90" s="17" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B90" s="15" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
+          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
@@ -10401,24 +10405,24 @@
       <c r="A91" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B91" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B91" s="17" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
+          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 1995be8</t>
+          <t>dr1v90 764f81d</t>
         </is>
       </c>
     </row>
@@ -10426,19 +10430,19 @@
       <c r="A92" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B92" s="20" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B92" s="15" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>D3;D4;D5</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
+          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
@@ -10451,20 +10455,24 @@
       <c r="A93" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B93" s="20" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C93" s="7" t="inlineStr"/>
+      <c r="B93" s="21" t="inlineStr">
+        <is>
+          <t>里程碑</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
+          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>dr1v90 task/d13-boot fdbb217</t>
         </is>
       </c>
     </row>
@@ -10472,20 +10480,24 @@
       <c r="A94" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B94" s="21" t="inlineStr">
-        <is>
-          <t>里程碑</t>
-        </is>
-      </c>
-      <c r="C94" s="7" t="inlineStr"/>
+      <c r="B94" s="17" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
+          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
         </is>
       </c>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -10493,20 +10505,24 @@
       <c r="A95" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B95" s="20" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C95" s="7" t="inlineStr"/>
+      <c r="B95" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
+          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_arch_common_front_display_backend.md</t>
+          <t>dr1v90 1995be8</t>
         </is>
       </c>
     </row>
@@ -10521,12 +10537,12 @@
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D3;D4;D5</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
+          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
@@ -10544,19 +10560,15 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C97" s="7" t="inlineStr">
-        <is>
-          <t>D11</t>
-        </is>
-      </c>
+      <c r="C97" s="7" t="inlineStr"/>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
+          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -10564,24 +10576,20 @@
       <c r="A98" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B98" s="20" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C98" s="7" t="inlineStr">
-        <is>
-          <t>D12;D13;D14</t>
-        </is>
-      </c>
+      <c r="B98" s="21" t="inlineStr">
+        <is>
+          <t>里程碑</t>
+        </is>
+      </c>
+      <c r="C98" s="7" t="inlineStr"/>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
+          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -10594,19 +10602,15 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C99" s="7" t="inlineStr">
-        <is>
-          <t>D13</t>
-        </is>
-      </c>
+      <c r="C99" s="7" t="inlineStr"/>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
+          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_arch_common_front_display_backend.md</t>
         </is>
       </c>
     </row>
@@ -10621,12 +10625,12 @@
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>D15;D16</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
         </is>
       </c>
       <c r="E100" s="7" t="inlineStr">
@@ -10646,17 +10650,17 @@
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>KR5.2</t>
+          <t>D11</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 49031f6</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -10664,19 +10668,19 @@
       <c r="A102" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B102" s="17" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B102" s="20" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D12;D13;D14</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
-          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
         </is>
       </c>
       <c r="E102" s="7" t="inlineStr">
@@ -10689,18 +10693,118 @@
       <c r="A103" s="19" t="n">
         <v>46308</v>
       </c>
-      <c r="B103" s="21" t="inlineStr">
+      <c r="B103" s="20" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C103" s="7" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
+      <c r="D103" s="7" t="inlineStr">
+        <is>
+          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
+        </is>
+      </c>
+      <c r="E103" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="19" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B104" s="20" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C104" s="7" t="inlineStr">
+        <is>
+          <t>D15;D16</t>
+        </is>
+      </c>
+      <c r="D104" s="7" t="inlineStr">
+        <is>
+          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+        </is>
+      </c>
+      <c r="E104" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="19" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B105" s="20" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C105" s="7" t="inlineStr">
+        <is>
+          <t>KR5.2</t>
+        </is>
+      </c>
+      <c r="D105" s="7" t="inlineStr">
+        <is>
+          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+        </is>
+      </c>
+      <c r="E105" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 49031f6</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="19" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B106" s="17" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C106" s="7" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="D106" s="7" t="inlineStr">
+        <is>
+          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+        </is>
+      </c>
+      <c r="E106" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="19" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B107" s="21" t="inlineStr">
         <is>
           <t>里程碑</t>
         </is>
       </c>
-      <c r="C103" s="7" t="inlineStr"/>
-      <c r="D103" s="7" t="inlineStr">
+      <c r="C107" s="7" t="inlineStr"/>
+      <c r="D107" s="7" t="inlineStr">
         <is>
           <t>显性目的进度看板第一版建立：10 个显性目的 + KR 趋势 + 燃起图 + 里程碑趋势</t>
         </is>
       </c>
-      <c r="E103" s="7" t="inlineStr">
+      <c r="E107" s="7" t="inlineStr">
         <is>
           <t>claude_memory/project_progress_dashboard.md</t>
         </is>
@@ -12230,9 +12334,9 @@
           <t>运维</t>
         </is>
       </c>
-      <c r="D26" s="17" t="inlineStr">
-        <is>
-          <t>🔄 进行中 / 未达标</t>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>✅ 达成当前期目标</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
@@ -12256,10 +12360,10 @@
         </is>
       </c>
       <c r="I26" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J26" s="19" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="K26" s="7" t="inlineStr">
         <is>
@@ -12275,18 +12379,18 @@
       <c r="N26" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O26" s="17" t="inlineStr">
-        <is>
-          <t>🔄</t>
+      <c r="O26" s="14" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="P26" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/rotor-ops 05c4231</t>
+          <t>dr1v90 dee9be6</t>
         </is>
       </c>
       <c r="Q26" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -12315,10 +12419,10 @@
         </is>
       </c>
       <c r="I27" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J27" s="19" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="K27" s="7" t="inlineStr">
         <is>
@@ -12334,18 +12438,18 @@
       <c r="N27" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O27" s="17" t="inlineStr">
-        <is>
-          <t>🔄</t>
+      <c r="O27" s="14" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="P27" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/rotor-ops 05c4231</t>
+          <t>dr1v90 dee9be6</t>
         </is>
       </c>
       <c r="Q27" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -14909,25 +15013,32 @@
       </c>
       <c r="C362" s="6" t="n"/>
       <c r="D362" s="8" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="E362" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F362" s="8" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="G362" s="6" t="n">
         <v>1</v>
       </c>
       <c r="H362" s="8" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="I362" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="363">
+      <c r="A363" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B363" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C363" s="6" t="n"/>
       <c r="D363" s="8" t="n">
         <v>46309</v>
       </c>
@@ -15010,25 +15121,32 @@
       </c>
       <c r="C379" s="6" t="n"/>
       <c r="D379" s="8" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="E379" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F379" s="8" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="G379" s="6" t="n">
         <v>1</v>
       </c>
       <c r="H379" s="8" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="I379" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="380">
+      <c r="A380" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B380" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C380" s="6" t="n"/>
       <c r="D380" s="8" t="n">
         <v>46309</v>
       </c>
@@ -15344,7 +15462,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -16034,15 +16152,17 @@
       <c r="E38" s="19" t="n">
         <v>46312</v>
       </c>
-      <c r="F38" s="19" t="n"/>
-      <c r="G38" s="17" t="inlineStr">
-        <is>
-          <t>🔄</t>
+      <c r="F38" s="19" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G38" s="14" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>7ef55e1 离线过; 上板 V3 待补测 (agent 已关, 开新的接)</t>
+          <t>合主线 dee9be6 (D7/D7b/D7c; 新克隆上板 V3N 连续 3 次 11/11 + V2 12/12, 离线回归 84 过)</t>
         </is>
       </c>
     </row>
@@ -16678,7 +16798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -19732,8 +19852,90 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="31" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B75" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>KR9.1</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>转子遥测可用 (1=可用)</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>是/否</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" s="7" t="inlineStr">
+        <is>
+          <t>V0 2047</t>
+        </is>
+      </c>
+      <c r="H75" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 dee9be6</t>
+        </is>
+      </c>
+      <c r="I75" s="7" t="inlineStr">
+        <is>
+          <t>povstat 遥测 + povnetd 状态上板可用</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="31" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B76" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>KR9.2</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>远程升级失败自动回滚 (1=有)</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>是/否</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>V0 2047</t>
+        </is>
+      </c>
+      <c r="H76" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 dee9be6</t>
+        </is>
+      </c>
+      <c r="I76" s="7" t="inlineStr">
+        <is>
+          <t>断网坏升级包连续 3 次自动回滚并按名字找回; 坏自检包回滚</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I74"/>
+  <autoFilter ref="A1:I76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>